<commit_message>
Update website with latest features
</commit_message>
<xml_diff>
--- a/server/data/database.xlsx
+++ b/server/data/database.xlsx
@@ -7,6 +7,9 @@
     <sheet name="Users" sheetId="2" r:id="rId2"/>
     <sheet name="Students" sheetId="3" r:id="rId3"/>
     <sheet name="Announcements" sheetId="4" r:id="rId4"/>
+    <sheet name="Baseline_Census" sheetId="5" r:id="rId5"/>
+    <sheet name="Enrollment Trends" sheetId="6" r:id="rId6"/>
+    <sheet name="Grade Breakdown" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -35,12 +38,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -404,149 +403,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A3:G65"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v xml:space="preserve">   SCHOOLS DIVISION OF PAMPANGA</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v xml:space="preserve">    VALDEZ ELEMENTARY SCHOOL</v>
-      </c>
-    </row>
-    <row r="3">
+    <row r="3" ht="26" customHeight="1">
       <c r="A3" t="str">
-        <v xml:space="preserve">    FLORIDABLANCA, PAMPANGA</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>SCHOOLS DIVISION OF PAMPANGA</v>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" t="str">
+        <v>VALDEZ ELEMENTARY SCHOOL</v>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" t="str">
+        <v>FLORIDABLANCA, PAMPANGA</v>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" t="str">
         <v>S.Y. 2025-2026</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" t="str">
         <v>GRADE LEVEL</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B8" t="str">
         <v>BOSY ENROLLMENT</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C8" t="str">
         <v>NUMBER OF REPEATERS</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D8" t="str">
         <v>NUMBER OF DROPOUTS</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E8" t="str">
         <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F8" t="str">
         <v>NUMBER OF SEATS</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G8" t="str">
         <v>NUMBER OF TEACHERS</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" t="str">
         <v>KINDER</v>
       </c>
-      <c r="B7">
+      <c r="B9">
         <v>67</v>
       </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7" t="str">
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="str">
         <v>3 (6x7)</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F9" t="str">
         <v>67</v>
       </c>
-      <c r="G7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
+      <c r="G9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" t="str">
         <v>GRADE 1</v>
       </c>
-      <c r="B8">
+      <c r="B10">
         <v>66</v>
       </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="str">
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="str">
         <v>2 (8x6)</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F10" t="str">
         <v>40 (2 seater desk)</v>
       </c>
-      <c r="G8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
+      <c r="G10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" t="str">
         <v>GRADE 2</v>
       </c>
-      <c r="B9">
+      <c r="B11">
         <v>71</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9" t="str">
-        <v>2 (7x6)</v>
-      </c>
-      <c r="F9" t="str">
-        <v>76</v>
-      </c>
-      <c r="G9">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>GRADE 3</v>
-      </c>
-      <c r="B10">
-        <v>74</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10" t="str">
-        <v>2 (9x7)</v>
-      </c>
-      <c r="F10" t="str">
-        <v>78</v>
-      </c>
-      <c r="G10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>GRADE 4</v>
-      </c>
-      <c r="B11">
-        <v>79</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -558,27 +521,27 @@
         <v>2 (7x6)</v>
       </c>
       <c r="F11" t="str">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G11">
         <v>2</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="17" customHeight="1">
       <c r="A12" t="str">
-        <v>GRADE 5</v>
+        <v>GRADE 3</v>
       </c>
       <c r="B12">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="str">
-        <v>2 (7x6)</v>
+        <v>2 (9x7)</v>
       </c>
       <c r="F12" t="str">
         <v>78</v>
@@ -587,201 +550,202 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="17" customHeight="1">
       <c r="A13" t="str">
-        <v>GRADE 6</v>
+        <v>GRADE 4</v>
       </c>
       <c r="B13">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="str">
         <v>2 (7x6)</v>
       </c>
       <c r="F13" t="str">
+        <v>82</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B14">
+        <v>77</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F14" t="str">
+        <v>78</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B15">
+        <v>68</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F15" t="str">
         <v>80</v>
       </c>
-      <c r="G13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
+      <c r="G15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" t="str">
         <v>RELIEVING TEACHER</v>
       </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v/>
-      </c>
-      <c r="G14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B15">
+      <c r="B17">
         <v>502</v>
       </c>
-      <c r="C15">
+      <c r="C17">
         <v>3</v>
       </c>
-      <c r="D15">
+      <c r="D17">
         <v>5</v>
       </c>
-      <c r="E15">
+      <c r="E17">
         <v>15</v>
       </c>
-      <c r="F15">
+      <c r="F17">
         <v>461</v>
       </c>
-      <c r="G15">
+      <c r="G17">
         <v>15</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="str">
+    <row r="18" ht="17" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" t="str">
         <v>S.Y. 2024-2025</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="str">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" t="str">
         <v>GRADE LEVEL</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B20" t="str">
         <v>BOSY ENROLLMENT</v>
       </c>
-      <c r="C18" t="str">
+      <c r="C20" t="str">
         <v>NUMBER OF REPEATERS</v>
       </c>
-      <c r="D18" t="str">
+      <c r="D20" t="str">
         <v>NUMBER OF DROPOUTS</v>
       </c>
-      <c r="E18" t="str">
+      <c r="E20" t="str">
         <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
       </c>
-      <c r="F18" t="str">
+      <c r="F20" t="str">
         <v>NUMBER OF SEATS</v>
       </c>
-      <c r="G18" t="str">
+      <c r="G20" t="str">
         <v>NUMBER OF TEACHERS</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="str">
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" t="str">
         <v>KINDER</v>
       </c>
-      <c r="B19">
+      <c r="B21">
         <v>64</v>
       </c>
-      <c r="C19">
-        <v>2</v>
-      </c>
-      <c r="D19">
-        <v>0</v>
-      </c>
-      <c r="E19" t="str">
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="str">
         <v>3 (6x7)</v>
       </c>
-      <c r="F19" t="str">
+      <c r="F21" t="str">
         <v>67</v>
       </c>
-      <c r="G19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
+      <c r="G21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" t="str">
         <v>GRADE 1</v>
       </c>
-      <c r="B20">
+      <c r="B22">
         <v>69</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20" t="str">
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="str">
         <v>2 (8x6)</v>
       </c>
-      <c r="F20" t="str">
+      <c r="F22" t="str">
         <v>40 (2 seater desk)</v>
       </c>
-      <c r="G20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
+      <c r="G22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" t="str">
         <v>GRADE 2</v>
       </c>
-      <c r="B21">
+      <c r="B23">
         <v>72</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
-      <c r="E21" t="str">
-        <v>2 (7x6)</v>
-      </c>
-      <c r="F21" t="str">
-        <v>76</v>
-      </c>
-      <c r="G21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>GRADE 3</v>
-      </c>
-      <c r="B22">
-        <v>75</v>
-      </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22" t="str">
-        <v>2 (9x7)</v>
-      </c>
-      <c r="F22" t="str">
-        <v>78</v>
-      </c>
-      <c r="G22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>GRADE 4</v>
-      </c>
-      <c r="B23">
-        <v>70</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -793,27 +757,27 @@
         <v>2 (7x6)</v>
       </c>
       <c r="F23" t="str">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G23">
         <v>2</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="17" customHeight="1">
       <c r="A24" t="str">
-        <v>GRADE 5</v>
+        <v>GRADE 3</v>
       </c>
       <c r="B24">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="str">
-        <v>2 (7x6)</v>
+        <v>2 (9x7)</v>
       </c>
       <c r="F24" t="str">
         <v>78</v>
@@ -822,15 +786,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="17" customHeight="1">
       <c r="A25" t="str">
-        <v>GRADE 6</v>
+        <v>GRADE 4</v>
       </c>
       <c r="B25">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -839,187 +803,188 @@
         <v>2 (7x6)</v>
       </c>
       <c r="F25" t="str">
+        <v>82</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B26">
+        <v>61</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F26" t="str">
+        <v>78</v>
+      </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B27">
+        <v>78</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F27" t="str">
         <v>80</v>
       </c>
-      <c r="G25">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
+      <c r="G27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" t="str">
         <v>RELIEVING TEACHER</v>
       </c>
-      <c r="B26" t="str">
-        <v/>
-      </c>
-      <c r="C26" t="str">
-        <v/>
-      </c>
-      <c r="D26" t="str">
-        <v/>
-      </c>
-      <c r="E26" t="str">
-        <v/>
-      </c>
-      <c r="F26" t="str">
-        <v/>
-      </c>
-      <c r="G26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B27">
+      <c r="B29">
         <v>489</v>
       </c>
-      <c r="C27">
+      <c r="C29">
         <v>4</v>
       </c>
-      <c r="D27">
-        <v>2</v>
-      </c>
-      <c r="E27">
+      <c r="D29">
+        <v>2</v>
+      </c>
+      <c r="E29">
         <v>15</v>
       </c>
-      <c r="F27">
+      <c r="F29">
         <v>461</v>
       </c>
-      <c r="G27">
+      <c r="G29">
         <v>14</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="str">
+    <row r="30" ht="17" customHeight="1"/>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" t="str">
         <v>S.Y. 2023-2024</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="str">
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" t="str">
         <v>GRADE LEVEL</v>
       </c>
-      <c r="B30" t="str">
+      <c r="B32" t="str">
         <v>BOSY ENROLLMENT</v>
       </c>
-      <c r="C30" t="str">
+      <c r="C32" t="str">
         <v>NUMBER OF REPEATERS</v>
       </c>
-      <c r="D30" t="str">
+      <c r="D32" t="str">
         <v>NUMBER OF DROPOUTS</v>
       </c>
-      <c r="E30" t="str">
+      <c r="E32" t="str">
         <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
       </c>
-      <c r="F30" t="str">
+      <c r="F32" t="str">
         <v>NUMBER OF SEATS</v>
       </c>
-      <c r="G30" t="str">
+      <c r="G32" t="str">
         <v>NUMBER OF TEACHERS</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="str">
+    <row r="33" ht="17" customHeight="1">
+      <c r="A33" t="str">
         <v>KINDER</v>
       </c>
-      <c r="B31">
+      <c r="B33">
         <v>78</v>
       </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="D31">
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
         <v>3</v>
       </c>
-      <c r="E31" t="str">
+      <c r="E33" t="str">
         <v>3 (6x7)</v>
       </c>
-      <c r="F31" t="str">
+      <c r="F33" t="str">
         <v>80</v>
       </c>
-      <c r="G31">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
+      <c r="G33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" ht="17" customHeight="1">
+      <c r="A34" t="str">
         <v>GRADE 1</v>
       </c>
-      <c r="B32">
+      <c r="B34">
         <v>76</v>
       </c>
-      <c r="C32">
-        <v>2</v>
-      </c>
-      <c r="D32">
-        <v>2</v>
-      </c>
-      <c r="E32" t="str">
+      <c r="C34">
+        <v>2</v>
+      </c>
+      <c r="D34">
+        <v>2</v>
+      </c>
+      <c r="E34" t="str">
         <v>2 (8x6)</v>
       </c>
-      <c r="F32" t="str">
+      <c r="F34" t="str">
         <v>40 (2 seater desk)</v>
       </c>
-      <c r="G32">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
+      <c r="G34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" t="str">
         <v>GRADE 2</v>
       </c>
-      <c r="B33">
+      <c r="B35">
         <v>62</v>
       </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33">
-        <v>0</v>
-      </c>
-      <c r="E33" t="str">
-        <v>2 (7x6)</v>
-      </c>
-      <c r="F33" t="str">
-        <v>76</v>
-      </c>
-      <c r="G33">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>GRADE 3</v>
-      </c>
-      <c r="B34">
-        <v>74</v>
-      </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-      <c r="D34">
-        <v>0</v>
-      </c>
-      <c r="E34" t="str">
-        <v>2 (9x7)</v>
-      </c>
-      <c r="F34" t="str">
-        <v>78</v>
-      </c>
-      <c r="G34">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>GRADE 4</v>
-      </c>
-      <c r="B35">
-        <v>64</v>
-      </c>
       <c r="C35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -1028,18 +993,18 @@
         <v>2 (7x6)</v>
       </c>
       <c r="F35" t="str">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="G35">
         <v>2</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="17" customHeight="1">
       <c r="A36" t="str">
-        <v>GRADE 5</v>
+        <v>GRADE 3</v>
       </c>
       <c r="B36">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -1048,7 +1013,7 @@
         <v>0</v>
       </c>
       <c r="E36" t="str">
-        <v>2 (7x6)</v>
+        <v>2 (9x7)</v>
       </c>
       <c r="F36" t="str">
         <v>78</v>
@@ -1057,224 +1022,225 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="17" customHeight="1">
       <c r="A37" t="str">
-        <v>GRADE 6</v>
+        <v>GRADE 4</v>
       </c>
       <c r="B37">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C37">
         <v>0</v>
       </c>
       <c r="D37">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E37" t="str">
         <v>2 (7x6)</v>
       </c>
       <c r="F37" t="str">
+        <v>67</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B38">
+        <v>77</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F38" t="str">
+        <v>78</v>
+      </c>
+      <c r="G38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B39">
+        <v>69</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>2</v>
+      </c>
+      <c r="E39" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F39" t="str">
         <v>80</v>
       </c>
-      <c r="G37">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
+      <c r="G39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" t="str">
         <v>RELIEVING TEACHER</v>
       </c>
-      <c r="B38" t="str">
-        <v/>
-      </c>
-      <c r="C38" t="str">
-        <v/>
-      </c>
-      <c r="D38" t="str">
-        <v/>
-      </c>
-      <c r="E38" t="str">
-        <v/>
-      </c>
-      <c r="F38" t="str">
-        <v/>
-      </c>
-      <c r="G38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B39">
+      <c r="B41">
         <v>500</v>
       </c>
-      <c r="C39">
+      <c r="C41">
         <v>3</v>
       </c>
-      <c r="D39">
+      <c r="D41">
         <v>7</v>
       </c>
-      <c r="E39">
+      <c r="E41">
         <v>15</v>
       </c>
-      <c r="F39">
+      <c r="F41">
         <v>461</v>
       </c>
-      <c r="G39">
+      <c r="G41">
         <v>15</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="str">
+    <row r="42" ht="17" customHeight="1"/>
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" t="str">
         <v>S.Y. 2022-2023</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="str">
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" t="str">
         <v>GRADE LEVEL</v>
       </c>
-      <c r="B42" t="str">
+      <c r="B44" t="str">
         <v>BOSY ENROLLMENT</v>
       </c>
-      <c r="C42" t="str">
+      <c r="C44" t="str">
         <v>NUMBER OF REPEATERS</v>
       </c>
-      <c r="D42" t="str">
+      <c r="D44" t="str">
         <v>NUMBER OF DROPOUTS</v>
       </c>
-      <c r="E42" t="str">
+      <c r="E44" t="str">
         <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
       </c>
-      <c r="F42" t="str">
+      <c r="F44" t="str">
         <v>NUMBER OF SEATS</v>
       </c>
-      <c r="G42" t="str">
+      <c r="G44" t="str">
         <v>NUMBER OF TEACHERS</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="str">
+    <row r="45" ht="17" customHeight="1">
+      <c r="A45" t="str">
         <v>KINDER</v>
       </c>
-      <c r="B43">
+      <c r="B45">
         <v>76</v>
       </c>
-      <c r="C43">
-        <v>0</v>
-      </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
-      <c r="E43" t="str">
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45" t="str">
         <v>3 (6x7)</v>
       </c>
-      <c r="F43" t="str">
+      <c r="F45" t="str">
         <v>80</v>
       </c>
-      <c r="G43">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
+      <c r="G45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" ht="17" customHeight="1">
+      <c r="A46" t="str">
         <v>GRADE 1</v>
       </c>
-      <c r="B44">
+      <c r="B46">
         <v>58</v>
       </c>
-      <c r="C44">
-        <v>0</v>
-      </c>
-      <c r="D44">
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
         <v>3</v>
       </c>
-      <c r="E44" t="str">
+      <c r="E46" t="str">
         <v>2 (8x6)</v>
       </c>
-      <c r="F44" t="str">
+      <c r="F46" t="str">
         <v>40 (2 seater desk)</v>
       </c>
-      <c r="G44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
+      <c r="G46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" ht="17" customHeight="1">
+      <c r="A47" t="str">
         <v>GRADE 2</v>
       </c>
-      <c r="B45">
+      <c r="B47">
         <v>72</v>
       </c>
-      <c r="C45">
-        <v>1</v>
-      </c>
-      <c r="D45">
-        <v>2</v>
-      </c>
-      <c r="E45" t="str">
-        <v>2 (7x6)</v>
-      </c>
-      <c r="F45" t="str">
-        <v>76</v>
-      </c>
-      <c r="G45">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>GRADE 3</v>
-      </c>
-      <c r="B46">
-        <v>54</v>
-      </c>
-      <c r="C46">
-        <v>0</v>
-      </c>
-      <c r="D46">
-        <v>0</v>
-      </c>
-      <c r="E46" t="str">
-        <v>2 (9x7)</v>
-      </c>
-      <c r="F46" t="str">
-        <v>54</v>
-      </c>
-      <c r="G46">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>GRADE 4</v>
-      </c>
-      <c r="B47">
-        <v>77</v>
-      </c>
       <c r="C47">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" t="str">
         <v>2 (7x6)</v>
       </c>
       <c r="F47" t="str">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G47">
         <v>2</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="17" customHeight="1">
       <c r="A48" t="str">
-        <v>GRADE 5</v>
+        <v>GRADE 3</v>
       </c>
       <c r="B48">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -1283,331 +1249,398 @@
         <v>0</v>
       </c>
       <c r="E48" t="str">
-        <v>2 (7x6)</v>
+        <v>2 (9x7)</v>
       </c>
       <c r="F48" t="str">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="G48">
         <v>2</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="17" customHeight="1">
       <c r="A49" t="str">
-        <v>GRADE 6</v>
+        <v>GRADE 4</v>
       </c>
       <c r="B49">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="C49">
         <v>0</v>
       </c>
       <c r="D49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" t="str">
         <v>2 (7x6)</v>
       </c>
       <c r="F49" t="str">
+        <v>80</v>
+      </c>
+      <c r="G49">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" ht="17" customHeight="1">
+      <c r="A50" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B50">
+        <v>70</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F50" t="str">
+        <v>78</v>
+      </c>
+      <c r="G50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" ht="17" customHeight="1">
+      <c r="A51" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B51">
+        <v>65</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F51" t="str">
         <v>67</v>
       </c>
-      <c r="G49">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
+      <c r="G51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" t="str">
         <v>RELIEVING TEACHER</v>
       </c>
-      <c r="B50" t="str">
-        <v/>
-      </c>
-      <c r="C50" t="str">
-        <v/>
-      </c>
-      <c r="D50" t="str">
-        <v/>
-      </c>
-      <c r="E50" t="str">
-        <v/>
-      </c>
-      <c r="F50" t="str">
-        <v/>
-      </c>
-      <c r="G50">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
+      <c r="B52" t="str">
+        <v/>
+      </c>
+      <c r="C52" t="str">
+        <v/>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B51">
+      <c r="B53">
         <v>472</v>
       </c>
-      <c r="C51">
-        <v>1</v>
-      </c>
-      <c r="D51">
+      <c r="C53">
+        <v>1</v>
+      </c>
+      <c r="D53">
         <v>7</v>
       </c>
-      <c r="E51">
+      <c r="E53">
         <v>15</v>
       </c>
-      <c r="F51">
+      <c r="F53">
         <v>461</v>
       </c>
-      <c r="G51">
+      <c r="G53">
         <v>15</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="str">
+    <row r="54" ht="17" customHeight="1"/>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" t="str">
         <v>S.Y. 2021-2022</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="str">
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" t="str">
         <v>GRADE LEVEL</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B56" t="str">
         <v>BOSY ENROLLMENT</v>
       </c>
-      <c r="C54" t="str">
+      <c r="C56" t="str">
         <v>NUMBER OF REPEATERS</v>
       </c>
-      <c r="D54" t="str">
+      <c r="D56" t="str">
         <v>NUMBER OF DROPOUTS</v>
       </c>
-      <c r="E54" t="str">
+      <c r="E56" t="str">
         <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
       </c>
-      <c r="F54" t="str">
+      <c r="F56" t="str">
         <v>NUMBER OF SEATS</v>
       </c>
-      <c r="G54" t="str">
+      <c r="G56" t="str">
         <v>NUMBER OF TEACHERS</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="str">
+    <row r="57" ht="17" customHeight="1">
+      <c r="A57" t="str">
         <v>KINDER</v>
       </c>
-      <c r="B55">
+      <c r="B57">
         <v>65</v>
       </c>
-      <c r="C55">
-        <v>0</v>
-      </c>
-      <c r="D55">
-        <v>0</v>
-      </c>
-      <c r="E55" t="str">
+      <c r="C57">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="str">
         <v>2 (6x7)</v>
       </c>
-      <c r="F55" t="str">
+      <c r="F57" t="str">
         <v>65</v>
       </c>
-      <c r="G55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
+      <c r="G57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" t="str">
         <v>GRADE 1</v>
       </c>
-      <c r="B56">
+      <c r="B58">
         <v>80</v>
       </c>
-      <c r="C56">
-        <v>2</v>
-      </c>
-      <c r="D56">
-        <v>1</v>
-      </c>
-      <c r="E56" t="str">
+      <c r="C58">
+        <v>2</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+      <c r="E58" t="str">
         <v>2 (8x6) and 1 (6x7)</v>
       </c>
-      <c r="F56" t="str">
+      <c r="F58" t="str">
         <v>40 (2 seater desk)</v>
-      </c>
-      <c r="G56">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>GRADE 2</v>
-      </c>
-      <c r="B57">
-        <v>57</v>
-      </c>
-      <c r="C57">
-        <v>0</v>
-      </c>
-      <c r="D57">
-        <v>1</v>
-      </c>
-      <c r="E57" t="str">
-        <v>2 (7x6)</v>
-      </c>
-      <c r="F57" t="str">
-        <v>59</v>
-      </c>
-      <c r="G57">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>GRADE 3</v>
-      </c>
-      <c r="B58">
-        <v>71</v>
-      </c>
-      <c r="C58">
-        <v>0</v>
-      </c>
-      <c r="D58">
-        <v>0</v>
-      </c>
-      <c r="E58" t="str">
-        <v>3 (9x7)</v>
-      </c>
-      <c r="F58" t="str">
-        <v>71</v>
       </c>
       <c r="G58">
         <v>3</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="17" customHeight="1">
       <c r="A59" t="str">
+        <v>GRADE 2</v>
+      </c>
+      <c r="B59">
+        <v>57</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F59" t="str">
+        <v>59</v>
+      </c>
+      <c r="G59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" ht="17" customHeight="1">
+      <c r="A60" t="str">
+        <v>GRADE 3</v>
+      </c>
+      <c r="B60">
+        <v>71</v>
+      </c>
+      <c r="C60">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="str">
+        <v>3 (9x7)</v>
+      </c>
+      <c r="F60" t="str">
+        <v>71</v>
+      </c>
+      <c r="G60">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61" ht="17" customHeight="1">
+      <c r="A61" t="str">
         <v>GRADE 4</v>
       </c>
-      <c r="B59">
+      <c r="B61">
         <v>70</v>
       </c>
-      <c r="C59">
-        <v>2</v>
-      </c>
-      <c r="D59">
-        <v>0</v>
-      </c>
-      <c r="E59" t="str">
+      <c r="C61">
+        <v>2</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="str">
         <v>3 (7x6)</v>
       </c>
-      <c r="F59" t="str">
+      <c r="F61" t="str">
         <v>70</v>
       </c>
-      <c r="G59">
+      <c r="G61">
         <v>3</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="str">
+    <row r="62" ht="17" customHeight="1">
+      <c r="A62" t="str">
         <v>GRADE 5</v>
       </c>
-      <c r="B60">
+      <c r="B62">
         <v>65</v>
       </c>
-      <c r="C60">
-        <v>0</v>
-      </c>
-      <c r="D60">
-        <v>0</v>
-      </c>
-      <c r="E60" t="str">
+      <c r="C62">
+        <v>0</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62" t="str">
         <v>2 (7x6)</v>
       </c>
-      <c r="F60" t="str">
+      <c r="F62" t="str">
         <v>65</v>
       </c>
-      <c r="G60">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
+      <c r="G62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" ht="17" customHeight="1">
+      <c r="A63" t="str">
         <v>GRADE 6</v>
       </c>
-      <c r="B61">
+      <c r="B63">
         <v>76</v>
       </c>
-      <c r="C61">
-        <v>0</v>
-      </c>
-      <c r="D61">
-        <v>0</v>
-      </c>
-      <c r="E61" t="str">
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="str">
         <v>2 (7x6)</v>
       </c>
-      <c r="F61" t="str">
+      <c r="F63" t="str">
         <v>76</v>
       </c>
-      <c r="G61">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
+      <c r="G63">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" t="str">
         <v>RELIEVING TEACHER</v>
       </c>
-      <c r="B62" t="str">
-        <v/>
-      </c>
-      <c r="C62" t="str">
-        <v/>
-      </c>
-      <c r="D62" t="str">
-        <v/>
-      </c>
-      <c r="E62" t="str">
-        <v/>
-      </c>
-      <c r="F62" t="str">
-        <v/>
-      </c>
-      <c r="G62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
+      <c r="B64" t="str">
+        <v/>
+      </c>
+      <c r="C64" t="str">
+        <v/>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B63">
+      <c r="B65">
         <v>484</v>
       </c>
-      <c r="C63">
+      <c r="C65">
         <v>4</v>
       </c>
-      <c r="D63">
-        <v>2</v>
-      </c>
-      <c r="E63">
+      <c r="D65">
+        <v>2</v>
+      </c>
+      <c r="E65">
         <v>15</v>
       </c>
-      <c r="F63">
+      <c r="F65">
         <v>461</v>
       </c>
-      <c r="G63">
+      <c r="G65">
         <v>16</v>
       </c>
     </row>
+    <row r="66" ht="17" customHeight="1"/>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A55:G55"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
+    <ignoredError numberStoredAsText="1" sqref="A3:G65"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" t="str">
         <v>id</v>
       </c>
@@ -1630,7 +1663,7 @@
         <v>gradeLevel</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" t="str">
         <v>A001</v>
       </c>
@@ -1650,7 +1683,7 @@
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" t="str">
         <v>T101</v>
       </c>
@@ -1673,7 +1706,7 @@
         <v>Grade 1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" t="str">
         <v>S201</v>
       </c>
@@ -1696,7 +1729,7 @@
         <v>Grade 1</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="18" customHeight="1">
       <c r="A5" t="str">
         <v>S8529_login</v>
       </c>
@@ -1719,7 +1752,7 @@
         <v>Grade 6</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" t="str">
         <v>S1965_login</v>
       </c>
@@ -1742,41 +1775,41 @@
         <v>Grade 6</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" t="str">
-        <v>S6428_login</v>
+        <v>T3243</v>
       </c>
       <c r="B7" t="str">
-        <v>Test Student</v>
+        <v>Ritch Nuguid</v>
       </c>
       <c r="C7" t="str">
-        <v>Student</v>
+        <v>Teacher</v>
       </c>
       <c r="D7" t="str">
-        <v>teststudent</v>
+        <v>ritchnuguid</v>
       </c>
       <c r="E7" t="str">
         <v>password123</v>
       </c>
       <c r="F7" t="str">
-        <v>Section A</v>
+        <v>Mabini</v>
       </c>
       <c r="G7" t="str">
-        <v>Kinder</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>Grade 1</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
       <c r="A8" t="str">
-        <v>T3243</v>
+        <v>T9288</v>
       </c>
       <c r="B8" t="str">
-        <v>Ritch Nuguid</v>
+        <v>laine perez</v>
       </c>
       <c r="C8" t="str">
         <v>Teacher</v>
       </c>
       <c r="D8" t="str">
-        <v>ritchnuguid</v>
+        <v>laineperez</v>
       </c>
       <c r="E8" t="str">
         <v>password123</v>
@@ -1788,41 +1821,98 @@
         <v>Grade 1</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" t="str">
-        <v>T9288</v>
+        <v>S3167_login</v>
       </c>
       <c r="B9" t="str">
-        <v>laine perez</v>
+        <v>Ritch Nuguid</v>
       </c>
       <c r="C9" t="str">
-        <v>Teacher</v>
+        <v>Student</v>
       </c>
       <c r="D9" t="str">
-        <v>laineperez</v>
+        <v>ritchnuguid</v>
       </c>
       <c r="E9" t="str">
         <v>password123</v>
       </c>
       <c r="F9" t="str">
+        <v>Aguinaldo</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Grade 4</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" t="str">
+        <v>S4723_login</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Ritch Nuguid</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Student</v>
+      </c>
+      <c r="D10" t="str">
+        <v>ritchnuguid</v>
+      </c>
+      <c r="E10" t="str">
+        <v>password123</v>
+      </c>
+      <c r="F10" t="str">
         <v>Mabini</v>
       </c>
-      <c r="G9" t="str">
+      <c r="G10" t="str">
         <v>Grade 1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF7"/>
+  <dimension ref="A1:AF8"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="25" max="25" width="12.83203125" customWidth="1"/>
+    <col min="26" max="26" width="12.83203125" customWidth="1"/>
+    <col min="27" max="27" width="12.83203125" customWidth="1"/>
+    <col min="28" max="28" width="12.83203125" customWidth="1"/>
+    <col min="29" max="29" width="12.83203125" customWidth="1"/>
+    <col min="30" max="30" width="12.83203125" customWidth="1"/>
+    <col min="31" max="31" width="12.83203125" customWidth="1"/>
+    <col min="32" max="32" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" t="str">
         <v>id</v>
       </c>
@@ -1920,7 +2010,7 @@
         <v>Makabayan_Q4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" t="str">
         <v>S201</v>
       </c>
@@ -1951,8 +2041,8 @@
       <c r="J2">
         <v>75</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
+      <c r="K2">
+        <v>85</v>
       </c>
       <c r="L2" t="str">
         <v/>
@@ -2018,7 +2108,7 @@
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" t="str">
         <v>S202</v>
       </c>
@@ -2116,7 +2206,7 @@
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" t="str">
         <v>S203</v>
       </c>
@@ -2214,7 +2304,7 @@
         <v/>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="18" customHeight="1">
       <c r="A5" t="str">
         <v>S8529</v>
       </c>
@@ -2312,7 +2402,7 @@
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" t="str">
         <v>S1965</v>
       </c>
@@ -2410,24 +2500,24 @@
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" t="str">
-        <v>S6428</v>
+        <v>S3167</v>
       </c>
       <c r="B7" t="str">
-        <v>10298976428</v>
+        <v>10282793167</v>
       </c>
       <c r="C7" t="str">
-        <v>Test Student</v>
+        <v>Ritch Nuguid</v>
       </c>
       <c r="D7" t="str">
         <v>Male</v>
       </c>
       <c r="E7" t="str">
-        <v>Kinder</v>
+        <v>Grade 4</v>
       </c>
       <c r="F7" t="str">
-        <v>Section A</v>
+        <v>Aguinaldo</v>
       </c>
       <c r="G7" t="str">
         <v>Enrolled</v>
@@ -2508,9 +2598,107 @@
         <v/>
       </c>
     </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" t="str">
+        <v>S4723</v>
+      </c>
+      <c r="B8" t="str">
+        <v>10283884723</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Ritch Nuguid</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Grade 1</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Mabini</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Enrolled</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+      <c r="AC8" t="str">
+        <v/>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
+      </c>
+      <c r="AE8" t="str">
+        <v/>
+      </c>
+      <c r="AF8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2518,8 +2706,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" t="str">
         <v>id</v>
       </c>
@@ -2536,7 +2731,7 @@
         <v>target</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2553,7 +2748,7 @@
         <v>All</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="18" customHeight="1">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2575,4 +2770,1527 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A3:G65"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" t="str">
+        <v>SCHOOLS DIVISION OF PAMPANGA</v>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" t="str">
+        <v>VALDEZ ELEMENTARY SCHOOL</v>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" t="str">
+        <v>FLORIDABLANCA, PAMPANGA</v>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" t="str">
+        <v>S.Y. 2025-2026</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" t="str">
+        <v>GRADE LEVEL</v>
+      </c>
+      <c r="B8" t="str">
+        <v>BOSY ENROLLMENT</v>
+      </c>
+      <c r="C8" t="str">
+        <v>NUMBER OF REPEATERS</v>
+      </c>
+      <c r="D8" t="str">
+        <v>NUMBER OF DROPOUTS</v>
+      </c>
+      <c r="E8" t="str">
+        <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
+      </c>
+      <c r="F8" t="str">
+        <v>NUMBER OF SEATS</v>
+      </c>
+      <c r="G8" t="str">
+        <v>NUMBER OF TEACHERS</v>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" t="str">
+        <v>KINDER</v>
+      </c>
+      <c r="B9">
+        <v>67</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="str">
+        <v>3 (6x7)</v>
+      </c>
+      <c r="F9" t="str">
+        <v>67</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" t="str">
+        <v>GRADE 1</v>
+      </c>
+      <c r="B10">
+        <v>65</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2 (8x6)</v>
+      </c>
+      <c r="F10" t="str">
+        <v>40 (2 seater desk)</v>
+      </c>
+      <c r="G10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" t="str">
+        <v>GRADE 2</v>
+      </c>
+      <c r="B11">
+        <v>71</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F11" t="str">
+        <v>76</v>
+      </c>
+      <c r="G11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" t="str">
+        <v>GRADE 3</v>
+      </c>
+      <c r="B12">
+        <v>74</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2 (9x7)</v>
+      </c>
+      <c r="F12" t="str">
+        <v>78</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" t="str">
+        <v>GRADE 4</v>
+      </c>
+      <c r="B13">
+        <v>78</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F13" t="str">
+        <v>82</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B14">
+        <v>77</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F14" t="str">
+        <v>78</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B15">
+        <v>66</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F15" t="str">
+        <v>80</v>
+      </c>
+      <c r="G15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" t="str">
+        <v>RELIEVING TEACHER</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B17">
+        <v>498</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+      <c r="F17">
+        <v>461</v>
+      </c>
+      <c r="G17">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" t="str">
+        <v>S.Y. 2024-2025</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" t="str">
+        <v>GRADE LEVEL</v>
+      </c>
+      <c r="B20" t="str">
+        <v>BOSY ENROLLMENT</v>
+      </c>
+      <c r="C20" t="str">
+        <v>NUMBER OF REPEATERS</v>
+      </c>
+      <c r="D20" t="str">
+        <v>NUMBER OF DROPOUTS</v>
+      </c>
+      <c r="E20" t="str">
+        <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
+      </c>
+      <c r="F20" t="str">
+        <v>NUMBER OF SEATS</v>
+      </c>
+      <c r="G20" t="str">
+        <v>NUMBER OF TEACHERS</v>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" t="str">
+        <v>KINDER</v>
+      </c>
+      <c r="B21">
+        <v>64</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="str">
+        <v>3 (6x7)</v>
+      </c>
+      <c r="F21" t="str">
+        <v>67</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" t="str">
+        <v>GRADE 1</v>
+      </c>
+      <c r="B22">
+        <v>69</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2 (8x6)</v>
+      </c>
+      <c r="F22" t="str">
+        <v>40 (2 seater desk)</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" t="str">
+        <v>GRADE 2</v>
+      </c>
+      <c r="B23">
+        <v>72</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F23" t="str">
+        <v>76</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" t="str">
+        <v>GRADE 3</v>
+      </c>
+      <c r="B24">
+        <v>75</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2 (9x7)</v>
+      </c>
+      <c r="F24" t="str">
+        <v>78</v>
+      </c>
+      <c r="G24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" t="str">
+        <v>GRADE 4</v>
+      </c>
+      <c r="B25">
+        <v>70</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F25" t="str">
+        <v>82</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B26">
+        <v>61</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F26" t="str">
+        <v>78</v>
+      </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B27">
+        <v>78</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F27" t="str">
+        <v>80</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" t="str">
+        <v>RELIEVING TEACHER</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B29">
+        <v>489</v>
+      </c>
+      <c r="C29">
+        <v>4</v>
+      </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
+      <c r="E29">
+        <v>15</v>
+      </c>
+      <c r="F29">
+        <v>461</v>
+      </c>
+      <c r="G29">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="17" customHeight="1"/>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" t="str">
+        <v>S.Y. 2023-2024</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" t="str">
+        <v>GRADE LEVEL</v>
+      </c>
+      <c r="B32" t="str">
+        <v>BOSY ENROLLMENT</v>
+      </c>
+      <c r="C32" t="str">
+        <v>NUMBER OF REPEATERS</v>
+      </c>
+      <c r="D32" t="str">
+        <v>NUMBER OF DROPOUTS</v>
+      </c>
+      <c r="E32" t="str">
+        <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
+      </c>
+      <c r="F32" t="str">
+        <v>NUMBER OF SEATS</v>
+      </c>
+      <c r="G32" t="str">
+        <v>NUMBER OF TEACHERS</v>
+      </c>
+    </row>
+    <row r="33" ht="17" customHeight="1">
+      <c r="A33" t="str">
+        <v>KINDER</v>
+      </c>
+      <c r="B33">
+        <v>78</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>3</v>
+      </c>
+      <c r="E33" t="str">
+        <v>3 (6x7)</v>
+      </c>
+      <c r="F33" t="str">
+        <v>80</v>
+      </c>
+      <c r="G33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" ht="17" customHeight="1">
+      <c r="A34" t="str">
+        <v>GRADE 1</v>
+      </c>
+      <c r="B34">
+        <v>76</v>
+      </c>
+      <c r="C34">
+        <v>2</v>
+      </c>
+      <c r="D34">
+        <v>2</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2 (8x6)</v>
+      </c>
+      <c r="F34" t="str">
+        <v>40 (2 seater desk)</v>
+      </c>
+      <c r="G34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" t="str">
+        <v>GRADE 2</v>
+      </c>
+      <c r="B35">
+        <v>62</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F35" t="str">
+        <v>76</v>
+      </c>
+      <c r="G35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" t="str">
+        <v>GRADE 3</v>
+      </c>
+      <c r="B36">
+        <v>74</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2 (9x7)</v>
+      </c>
+      <c r="F36" t="str">
+        <v>78</v>
+      </c>
+      <c r="G36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" t="str">
+        <v>GRADE 4</v>
+      </c>
+      <c r="B37">
+        <v>64</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F37" t="str">
+        <v>67</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B38">
+        <v>77</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F38" t="str">
+        <v>78</v>
+      </c>
+      <c r="G38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B39">
+        <v>69</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>2</v>
+      </c>
+      <c r="E39" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F39" t="str">
+        <v>80</v>
+      </c>
+      <c r="G39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" t="str">
+        <v>RELIEVING TEACHER</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B41">
+        <v>500</v>
+      </c>
+      <c r="C41">
+        <v>3</v>
+      </c>
+      <c r="D41">
+        <v>7</v>
+      </c>
+      <c r="E41">
+        <v>15</v>
+      </c>
+      <c r="F41">
+        <v>461</v>
+      </c>
+      <c r="G41">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1"/>
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" t="str">
+        <v>S.Y. 2022-2023</v>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" t="str">
+        <v>GRADE LEVEL</v>
+      </c>
+      <c r="B44" t="str">
+        <v>BOSY ENROLLMENT</v>
+      </c>
+      <c r="C44" t="str">
+        <v>NUMBER OF REPEATERS</v>
+      </c>
+      <c r="D44" t="str">
+        <v>NUMBER OF DROPOUTS</v>
+      </c>
+      <c r="E44" t="str">
+        <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
+      </c>
+      <c r="F44" t="str">
+        <v>NUMBER OF SEATS</v>
+      </c>
+      <c r="G44" t="str">
+        <v>NUMBER OF TEACHERS</v>
+      </c>
+    </row>
+    <row r="45" ht="17" customHeight="1">
+      <c r="A45" t="str">
+        <v>KINDER</v>
+      </c>
+      <c r="B45">
+        <v>76</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45" t="str">
+        <v>3 (6x7)</v>
+      </c>
+      <c r="F45" t="str">
+        <v>80</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" ht="17" customHeight="1">
+      <c r="A46" t="str">
+        <v>GRADE 1</v>
+      </c>
+      <c r="B46">
+        <v>58</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>3</v>
+      </c>
+      <c r="E46" t="str">
+        <v>2 (8x6)</v>
+      </c>
+      <c r="F46" t="str">
+        <v>40 (2 seater desk)</v>
+      </c>
+      <c r="G46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" ht="17" customHeight="1">
+      <c r="A47" t="str">
+        <v>GRADE 2</v>
+      </c>
+      <c r="B47">
+        <v>72</v>
+      </c>
+      <c r="C47">
+        <v>1</v>
+      </c>
+      <c r="D47">
+        <v>2</v>
+      </c>
+      <c r="E47" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F47" t="str">
+        <v>76</v>
+      </c>
+      <c r="G47">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" ht="17" customHeight="1">
+      <c r="A48" t="str">
+        <v>GRADE 3</v>
+      </c>
+      <c r="B48">
+        <v>54</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48" t="str">
+        <v>2 (9x7)</v>
+      </c>
+      <c r="F48" t="str">
+        <v>54</v>
+      </c>
+      <c r="G48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" ht="17" customHeight="1">
+      <c r="A49" t="str">
+        <v>GRADE 4</v>
+      </c>
+      <c r="B49">
+        <v>77</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>1</v>
+      </c>
+      <c r="E49" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F49" t="str">
+        <v>80</v>
+      </c>
+      <c r="G49">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" ht="17" customHeight="1">
+      <c r="A50" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B50">
+        <v>70</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F50" t="str">
+        <v>78</v>
+      </c>
+      <c r="G50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" ht="17" customHeight="1">
+      <c r="A51" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B51">
+        <v>65</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F51" t="str">
+        <v>67</v>
+      </c>
+      <c r="G51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" t="str">
+        <v>RELIEVING TEACHER</v>
+      </c>
+      <c r="B52" t="str">
+        <v/>
+      </c>
+      <c r="C52" t="str">
+        <v/>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B53">
+        <v>472</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+      <c r="D53">
+        <v>7</v>
+      </c>
+      <c r="E53">
+        <v>15</v>
+      </c>
+      <c r="F53">
+        <v>461</v>
+      </c>
+      <c r="G53">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" ht="17" customHeight="1"/>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" t="str">
+        <v>S.Y. 2021-2022</v>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" t="str">
+        <v>GRADE LEVEL</v>
+      </c>
+      <c r="B56" t="str">
+        <v>BOSY ENROLLMENT</v>
+      </c>
+      <c r="C56" t="str">
+        <v>NUMBER OF REPEATERS</v>
+      </c>
+      <c r="D56" t="str">
+        <v>NUMBER OF DROPOUTS</v>
+      </c>
+      <c r="E56" t="str">
+        <v>NUMBER OF FUNCTIONAL CLASSROOMS</v>
+      </c>
+      <c r="F56" t="str">
+        <v>NUMBER OF SEATS</v>
+      </c>
+      <c r="G56" t="str">
+        <v>NUMBER OF TEACHERS</v>
+      </c>
+    </row>
+    <row r="57" ht="17" customHeight="1">
+      <c r="A57" t="str">
+        <v>KINDER</v>
+      </c>
+      <c r="B57">
+        <v>65</v>
+      </c>
+      <c r="C57">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="str">
+        <v>2 (6x7)</v>
+      </c>
+      <c r="F57" t="str">
+        <v>65</v>
+      </c>
+      <c r="G57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" t="str">
+        <v>GRADE 1</v>
+      </c>
+      <c r="B58">
+        <v>80</v>
+      </c>
+      <c r="C58">
+        <v>2</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+      <c r="E58" t="str">
+        <v>2 (8x6) and 1 (6x7)</v>
+      </c>
+      <c r="F58" t="str">
+        <v>40 (2 seater desk)</v>
+      </c>
+      <c r="G58">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" ht="17" customHeight="1">
+      <c r="A59" t="str">
+        <v>GRADE 2</v>
+      </c>
+      <c r="B59">
+        <v>57</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F59" t="str">
+        <v>59</v>
+      </c>
+      <c r="G59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" ht="17" customHeight="1">
+      <c r="A60" t="str">
+        <v>GRADE 3</v>
+      </c>
+      <c r="B60">
+        <v>71</v>
+      </c>
+      <c r="C60">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="str">
+        <v>3 (9x7)</v>
+      </c>
+      <c r="F60" t="str">
+        <v>71</v>
+      </c>
+      <c r="G60">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61" ht="17" customHeight="1">
+      <c r="A61" t="str">
+        <v>GRADE 4</v>
+      </c>
+      <c r="B61">
+        <v>70</v>
+      </c>
+      <c r="C61">
+        <v>2</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="str">
+        <v>3 (7x6)</v>
+      </c>
+      <c r="F61" t="str">
+        <v>70</v>
+      </c>
+      <c r="G61">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" ht="17" customHeight="1">
+      <c r="A62" t="str">
+        <v>GRADE 5</v>
+      </c>
+      <c r="B62">
+        <v>65</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F62" t="str">
+        <v>65</v>
+      </c>
+      <c r="G62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" ht="17" customHeight="1">
+      <c r="A63" t="str">
+        <v>GRADE 6</v>
+      </c>
+      <c r="B63">
+        <v>76</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="str">
+        <v>2 (7x6)</v>
+      </c>
+      <c r="F63" t="str">
+        <v>76</v>
+      </c>
+      <c r="G63">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" t="str">
+        <v>RELIEVING TEACHER</v>
+      </c>
+      <c r="B64" t="str">
+        <v/>
+      </c>
+      <c r="C64" t="str">
+        <v/>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B65">
+        <v>484</v>
+      </c>
+      <c r="C65">
+        <v>4</v>
+      </c>
+      <c r="D65">
+        <v>2</v>
+      </c>
+      <c r="E65">
+        <v>15</v>
+      </c>
+      <c r="F65">
+        <v>461</v>
+      </c>
+      <c r="G65">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" ht="17" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A55:G55"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A3:G65"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" t="str">
+        <v>School Year</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Total Students</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Total Repeaters</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Total Dropouts</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Total Teachers</v>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="str">
+        <v>S.Y. 2025-2026</v>
+      </c>
+      <c r="B2">
+        <v>502</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" t="str">
+        <v>S.Y. 2024-2025</v>
+      </c>
+      <c r="B3">
+        <v>489</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" t="str">
+        <v>S.Y. 2023-2024</v>
+      </c>
+      <c r="B4">
+        <v>500</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>7</v>
+      </c>
+      <c r="E4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" t="str">
+        <v>S.Y. 2022-2023</v>
+      </c>
+      <c r="B5">
+        <v>472</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" t="str">
+        <v>S.Y. 2021-2022</v>
+      </c>
+      <c r="B6">
+        <v>484</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H6"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" t="str">
+        <v>School Year</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Kinder</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Grade 1</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Grade 2</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Grade 3</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Grade 4</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Grade 5</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Grade 6</v>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="str">
+        <v>S.Y. 2025-2026</v>
+      </c>
+      <c r="B2">
+        <v>67</v>
+      </c>
+      <c r="C2">
+        <v>66</v>
+      </c>
+      <c r="D2">
+        <v>71</v>
+      </c>
+      <c r="E2">
+        <v>74</v>
+      </c>
+      <c r="F2">
+        <v>79</v>
+      </c>
+      <c r="G2">
+        <v>77</v>
+      </c>
+      <c r="H2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" t="str">
+        <v>S.Y. 2024-2025</v>
+      </c>
+      <c r="B3">
+        <v>64</v>
+      </c>
+      <c r="C3">
+        <v>69</v>
+      </c>
+      <c r="D3">
+        <v>72</v>
+      </c>
+      <c r="E3">
+        <v>75</v>
+      </c>
+      <c r="F3">
+        <v>70</v>
+      </c>
+      <c r="G3">
+        <v>61</v>
+      </c>
+      <c r="H3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" t="str">
+        <v>S.Y. 2023-2024</v>
+      </c>
+      <c r="B4">
+        <v>78</v>
+      </c>
+      <c r="C4">
+        <v>76</v>
+      </c>
+      <c r="D4">
+        <v>62</v>
+      </c>
+      <c r="E4">
+        <v>74</v>
+      </c>
+      <c r="F4">
+        <v>64</v>
+      </c>
+      <c r="G4">
+        <v>77</v>
+      </c>
+      <c r="H4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" t="str">
+        <v>S.Y. 2022-2023</v>
+      </c>
+      <c r="B5">
+        <v>76</v>
+      </c>
+      <c r="C5">
+        <v>58</v>
+      </c>
+      <c r="D5">
+        <v>72</v>
+      </c>
+      <c r="E5">
+        <v>54</v>
+      </c>
+      <c r="F5">
+        <v>77</v>
+      </c>
+      <c r="G5">
+        <v>70</v>
+      </c>
+      <c r="H5">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" t="str">
+        <v>S.Y. 2021-2022</v>
+      </c>
+      <c r="B6">
+        <v>65</v>
+      </c>
+      <c r="C6">
+        <v>80</v>
+      </c>
+      <c r="D6">
+        <v>57</v>
+      </c>
+      <c r="E6">
+        <v>71</v>
+      </c>
+      <c r="F6">
+        <v>70</v>
+      </c>
+      <c r="G6">
+        <v>65</v>
+      </c>
+      <c r="H6">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>